<commit_message>
Add WIP BOL generator and template updates
Introduces a new `bol_generator_wip.js` workflow to parse CSV orders, fetch shipment details from Acumatica, populate Master/Supplemental BOL sheets in Excel, and export the result to PDF via LibreOffice. Adds a new `.env` template with Acumatica, file path, and LibreOffice configuration placeholders. Updates `BOL_Template.xlsx` and `mapping.xlsx` to align the template and field mapping with the new generation flow.
</commit_message>
<xml_diff>
--- a/Istar_Development/Projects/BOL_Generation/Code/templates/BOL_Template.xlsx
+++ b/Istar_Development/Projects/BOL_Generation/Code/templates/BOL_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Procomm\Documents\GitHub\Acumatica_Customizations_and_Packages\Istar_Development\Projects\BOL_Generation\Code\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E097467-11F9-48A5-9D0E-F74C65F0CAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D66ACD8-23A7-4AB8-8E70-7666E918D329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{888CA347-7849-4038-B8EE-FAC87BA1B844}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="83">
   <si>
     <t>SHIP FROM</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>Address: 910 Nestle Way</t>
+  </si>
+  <si>
+    <t>BX</t>
   </si>
   <si>
     <t>Page 1 of 2</t>
@@ -4486,7 +4489,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="436" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" s="437"/>
       <c r="C1" s="279" t="s">
@@ -4501,7 +4504,7 @@
       <c r="J1" s="279"/>
       <c r="K1" s="279"/>
       <c r="L1" s="280" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="M1" s="281"/>
     </row>
@@ -4517,7 +4520,7 @@
       <c r="G2" s="277"/>
       <c r="H2" s="278"/>
       <c r="I2" s="282" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J2" s="283"/>
       <c r="K2" s="283"/>
@@ -4526,7 +4529,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="264" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" s="265"/>
       <c r="C3" s="265"/>
@@ -4543,7 +4546,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="264" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="265"/>
       <c r="C4" s="265"/>
@@ -4560,7 +4563,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="264" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B5" s="265"/>
       <c r="C5" s="265"/>
@@ -4606,7 +4609,7 @@
       <c r="G7" s="277"/>
       <c r="H7" s="278"/>
       <c r="I7" s="86" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J7" s="87"/>
       <c r="K7" s="88"/>
@@ -4615,7 +4618,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="300" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="301"/>
       <c r="C8" s="301"/>
@@ -4646,7 +4649,7 @@
       <c r="G9" s="301"/>
       <c r="H9" s="304"/>
       <c r="I9" s="90" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J9" s="91"/>
       <c r="K9" s="91"/>
@@ -4655,7 +4658,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="300" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B10" s="301"/>
       <c r="C10" s="301"/>
@@ -4665,7 +4668,7 @@
       <c r="G10" s="301"/>
       <c r="H10" s="304"/>
       <c r="I10" s="92" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J10" s="93"/>
       <c r="K10" s="93"/>
@@ -4686,7 +4689,7 @@
       <c r="G11" s="290"/>
       <c r="H11" s="85"/>
       <c r="I11" s="95" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J11" s="96"/>
       <c r="K11" s="96"/>
@@ -4765,7 +4768,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="98" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B16" s="99"/>
       <c r="C16" s="99"/>
@@ -4775,7 +4778,7 @@
       <c r="G16" s="373"/>
       <c r="H16" s="374"/>
       <c r="I16" s="325" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J16" s="326"/>
       <c r="K16" s="326"/>
@@ -6408,7 +6411,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="436" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="437"/>
       <c r="C1" s="279" t="s">
@@ -6423,7 +6426,7 @@
       <c r="J1" s="279"/>
       <c r="K1" s="279"/>
       <c r="L1" s="280" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M1" s="281"/>
     </row>
@@ -7601,20 +7604,20 @@
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="241"/>
       <c r="C1" s="241"/>
       <c r="F1" s="40"/>
       <c r="G1" s="40" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H1" s="40"/>
       <c r="I1" s="40"/>
       <c r="J1" s="41"/>
       <c r="K1" s="41"/>
       <c r="L1" s="246" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M1" s="247"/>
     </row>
@@ -7637,7 +7640,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="207" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" s="208"/>
       <c r="C3" s="208"/>
@@ -7647,7 +7650,7 @@
       <c r="G3" s="208"/>
       <c r="H3" s="209"/>
       <c r="I3" s="45" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J3" s="43"/>
       <c r="K3" s="46"/>
@@ -7656,7 +7659,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="207" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="208"/>
       <c r="C4" s="208"/>
@@ -7673,7 +7676,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="207" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B5" s="208"/>
       <c r="C5" s="208"/>
@@ -7719,7 +7722,7 @@
       <c r="G7" s="259"/>
       <c r="H7" s="260"/>
       <c r="I7" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J7" s="50"/>
       <c r="K7" s="51"/>
@@ -7753,7 +7756,7 @@
       </c>
       <c r="H9" s="56"/>
       <c r="I9" s="57" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J9" s="58"/>
       <c r="K9" s="58"/>
@@ -7762,7 +7765,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="59" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C10" s="236"/>
       <c r="D10" s="236"/>
@@ -7771,7 +7774,7 @@
       <c r="G10" s="236"/>
       <c r="H10" s="56"/>
       <c r="I10" s="60" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J10" s="61"/>
       <c r="K10" s="61"/>
@@ -7792,7 +7795,7 @@
       <c r="G11" s="252"/>
       <c r="H11" s="48"/>
       <c r="I11" s="239" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J11" s="240"/>
       <c r="K11" s="63"/>
@@ -7879,7 +7882,7 @@
       <c r="G16" s="32"/>
       <c r="H16" s="33"/>
       <c r="I16" s="230" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J16" s="231"/>
       <c r="K16" s="231"/>
@@ -7888,7 +7891,7 @@
     </row>
     <row r="17" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="34" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B17" s="35"/>
       <c r="C17" s="35"/>
@@ -8225,13 +8228,17 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" s="66"/>
-      <c r="B34" s="10"/>
+      <c r="B34" s="10" t="s">
+        <v>60</v>
+      </c>
       <c r="C34" s="9"/>
-      <c r="D34" s="65"/>
+      <c r="D34" s="65" t="s">
+        <v>60</v>
+      </c>
       <c r="E34" s="9"/>
       <c r="F34" s="10"/>
       <c r="G34" s="161" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H34" s="162"/>
       <c r="I34" s="162"/>

</xml_diff>

<commit_message>
Remove non-printable sheets from BOL output
Update BOL generation to delete reference/template worksheets instead of hiding them so LibreOffice headless PDF conversion won’t include hidden sheets. ADDRESS, Customer Order Info, and Supplemental_BOL are always removed, and Supplemental_Master_BOL is removed when there are no overflow orders. The BOL template workbook was updated to align with this output behavior.
</commit_message>
<xml_diff>
--- a/Istar_Development/Projects/BOL_Generation/Code/templates/BOL_Template.xlsx
+++ b/Istar_Development/Projects/BOL_Generation/Code/templates/BOL_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Procomm\Documents\GitHub\Acumatica_Customizations_and_Packages\Istar_Development\Projects\BOL_Generation\Code\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC6B49A3-2085-4DF2-A6B3-2CB1712A114E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1FD027-D5F0-4466-A1F9-03A693F9CFF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{888CA347-7849-4038-B8EE-FAC87BA1B844}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{888CA347-7849-4038-B8EE-FAC87BA1B844}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterBOL" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="83">
   <si>
     <t>SHIP FROM</t>
   </si>
@@ -5068,7 +5068,9 @@
       <c r="A34" s="83"/>
       <c r="B34" s="80"/>
       <c r="C34" s="81"/>
-      <c r="D34" s="80"/>
+      <c r="D34" s="80" t="s">
+        <v>60</v>
+      </c>
       <c r="E34" s="81"/>
       <c r="F34" s="80"/>
       <c r="G34" s="283"/>

</xml_diff>

<commit_message>
Update BOL template spreadsheets
Refresh the BOL generation Excel assets by updating both `BOL_Template.xlsx` and `mapping.xlsx`. This keeps the generated bill of lading output aligned with the latest template layout and field mapping configuration.
</commit_message>
<xml_diff>
--- a/Istar_Development/Projects/BOL_Generation/Code/templates/BOL_Template.xlsx
+++ b/Istar_Development/Projects/BOL_Generation/Code/templates/BOL_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Procomm\Documents\GitHub\Acumatica_Customizations_and_Packages\Istar_Development\Projects\BOL_Generation\Code\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7014F9B9-38B0-48A2-B7A1-405CAF8EE714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0689B93-5F4C-41BC-9FEE-95ABBBE7B28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2640" yWindow="2640" windowWidth="28800" windowHeight="15345" xr2:uid="{888CA347-7849-4038-B8EE-FAC87BA1B844}"/>
   </bookViews>
@@ -2130,10 +2130,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="33" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="29" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>